<commit_message>
fix: Partner Payouts 이중 곱셈 버그 수정 + Schedule 탭 2행 재설계 + Hero 완성 (5/19)
- Partner Payouts: base_price 이중 곱셈 버그 수정 (₩882M→정상 계산)
  - base_price는 이미 총액(단가×qty bake-in) — ×quantity 재곱 제거
  - Trip Services: base_price / contractedQty × scheduledDays 로 실제 일수 반영
- Partner Payouts: Reset 기능 추가 (파트너 이름 확인 후 delete → 재입력)
- Partner Payouts: KRW 표시 통일, 단가×qty 분해 표시 (₩1,500,000 × 3d = ₩4,500,000)
- 호텔 단위: variant_label_snapshot "night" 포함 여부로 'pax'→'d' 교정
- Overview: Earnings 음수 시 빨간색 표시
- ScheduleDocument: showInternalNotes 활성 시 Admin:/Agent: 2행 탭 구조
  - 행 클릭 = viewerMode + activeGroupId 동시 설정
  - effectiveShowInternal = showInternalNotes && viewerMode === 'admin'
- CaseHeroAction: awaiting_settlement Agent/Admin 케이스 추가
- CaseHeroAction: noPrefix prop으로 completed "Next·" prefix 제거

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/products_master_Hong_260513_K_Wellness_Spa 수정_v2.xlsx
+++ b/data/products_master_Hong_260513_K_Wellness_Spa 수정_v2.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3B22C8-FD32-4AF7-86B3-E5330835D08F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7998B32B-6E2C-439E-B422-D7C76707AADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="K-Medical" sheetId="1" r:id="rId1"/>
@@ -8511,7 +8511,9 @@
       <c r="J8" s="2" t="s">
         <v>742</v>
       </c>
-      <c r="K8" s="10"/>
+      <c r="K8" s="10">
+        <v>1000000</v>
+      </c>
       <c r="L8" s="2" t="s">
         <v>31</v>
       </c>

</xml_diff>